<commit_message>
Update 2 Juni 2026
- Persepsi (naik/turun)
- Delay Google News
</commit_message>
<xml_diff>
--- a/Kata Kunci.xlsx
+++ b/Kata Kunci.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Argo\!!2026\AI\Antigravity\berita\Web-Scraping-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A204505-CF1C-4514-9374-40474075A862}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54C2440A-4011-4023-A5A2-2CB702E21643}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7695" xr2:uid="{A8968677-769D-4485-84B0-F2D4272DC42E}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7695" activeTab="1" xr2:uid="{A8968677-769D-4485-84B0-F2D4272DC42E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="keyword" sheetId="1" r:id="rId1"/>
+    <sheet name="persepsi" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="87">
   <si>
     <t>Organisasi Kemasyarakatan</t>
   </si>
@@ -202,6 +203,90 @@
   </si>
   <si>
     <t>Tsunami</t>
+  </si>
+  <si>
+    <t>naik</t>
+  </si>
+  <si>
+    <t>turun</t>
+  </si>
+  <si>
+    <t>bertambah</t>
+  </si>
+  <si>
+    <t>berkurang</t>
+  </si>
+  <si>
+    <t>meningkat</t>
+  </si>
+  <si>
+    <t>menurun</t>
+  </si>
+  <si>
+    <t>tumbuh</t>
+  </si>
+  <si>
+    <t>melambat</t>
+  </si>
+  <si>
+    <t>lebih besar</t>
+  </si>
+  <si>
+    <t>lebih kecil</t>
+  </si>
+  <si>
+    <t>lebih banyak</t>
+  </si>
+  <si>
+    <t>lebih sedikit</t>
+  </si>
+  <si>
+    <t>percepatan</t>
+  </si>
+  <si>
+    <t>perlambatan</t>
+  </si>
+  <si>
+    <t>melesat</t>
+  </si>
+  <si>
+    <t>anjlok</t>
+  </si>
+  <si>
+    <t>lebih cepat</t>
+  </si>
+  <si>
+    <t>lebih lambat</t>
+  </si>
+  <si>
+    <t>lebih tinggi</t>
+  </si>
+  <si>
+    <t>lebih rendah</t>
+  </si>
+  <si>
+    <t>lebih luas</t>
+  </si>
+  <si>
+    <t>lebih sempit</t>
+  </si>
+  <si>
+    <t>meluas</t>
+  </si>
+  <si>
+    <t>menyempit</t>
+  </si>
+  <si>
+    <t>lebih kuat</t>
+  </si>
+  <si>
+    <t>lebih lemah</t>
+  </si>
+  <si>
+    <t>menguat</t>
+  </si>
+  <si>
+    <t>melemah</t>
   </si>
 </sst>
 </file>
@@ -770,4 +855,137 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{733CDB76-AE75-4AF6-86E2-6980EF40DE66}">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>